<commit_message>
Fix crashes and rendering defects found in generation review
- xlsx: milestone/note landing inside a merged bar no longer crashes
  (write via merge anchor; milestone text is appended to the bar label)
- xlsx: "today" line survives merged bars (openpyxl rewrites merged-range
  borders from the anchor cell on save); skipped honestly when today falls
  inside a bar instead of drawing at the wrong edge
- xlsx: bar borders use line colors so stacked same-style bars don't fuse
- pptx: warn on milestone overlaps; reserve milestone label weeks
- common: warn when bar start/end are reversed instead of silent swap
- sample/schema: MPV->MVP typo, shorten bar label that got truncated,
  document overlap degradation and today-inside-bar limitation
- SKILL.md: sync rows-per-slide with code (15)
- remove stale preview PNGs; rebuild demos, .skill and full.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap_demo.xlsx
+++ b/roadmap_demo.xlsx
@@ -144,16 +144,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00F5A623"/>
+        <color rgb="00C77F00"/>
       </left>
       <right style="thin">
-        <color rgb="00F5A623"/>
+        <color rgb="00C77F00"/>
       </right>
       <top style="thin">
-        <color rgb="00F5A623"/>
+        <color rgb="00C77F00"/>
       </top>
       <bottom style="thin">
-        <color rgb="00F5A623"/>
+        <color rgb="00C77F00"/>
       </bottom>
     </border>
     <border>
@@ -202,30 +202,30 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00FBEAB6"/>
+        <color rgb="00E0C878"/>
       </left>
       <right style="thin">
-        <color rgb="00FBEAB6"/>
+        <color rgb="00E0C878"/>
       </right>
       <top style="thin">
-        <color rgb="00FBEAB6"/>
+        <color rgb="00E0C878"/>
       </top>
       <bottom style="thin">
-        <color rgb="00FBEAB6"/>
+        <color rgb="00E0C878"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </left>
       <right style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </right>
       <top style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </top>
       <bottom style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </bottom>
     </border>
     <border>
@@ -244,16 +244,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </left>
       <right style="medium">
         <color rgb="002E7D32"/>
       </right>
       <top style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </top>
       <bottom style="thin">
-        <color rgb="00FFF176"/>
+        <color rgb="00D4C24A"/>
       </bottom>
     </border>
   </borders>
@@ -302,10 +302,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -730,7 +730,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>MPV — синий</t>
+          <t>MVP — синий</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,8 @@
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>КАФО агента (Интеграция, взаимодействие)
-(Д. Шатыр)</t>
+(Д. Шатыр)
+Сервисы: CTL, ClickHouse, СберЧат, ЛДБР, IDP</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -913,7 +914,7 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Согласование</t>
+          <t>Согласов.</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -974,7 +975,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>🗨</t>
+          <t>💬</t>
         </is>
       </c>
       <c r="I9" s="10" t="n"/>
@@ -1155,7 +1156,7 @@
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>🗨</t>
+          <t>💬</t>
         </is>
       </c>
       <c r="F15" s="10" t="n"/>
@@ -1173,7 +1174,8 @@
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Интеграция
-(С. Славский ?)</t>
+(С. Славский ?)
+Сервисы: CTL, СберЧат, ClickHouse</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1253,7 +1255,8 @@
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Интеграция с IDP (RAG)
-(С. Славский ?)</t>
+(С. Славский ?)
+Сервисы: IDP</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1291,7 +1294,7 @@
       <c r="E20" s="10" t="n"/>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>🗨</t>
+          <t>💬</t>
         </is>
       </c>
       <c r="G20" s="10" t="n"/>

</xml_diff>